<commit_message>
Fix financial model logic: improve tenancy data parsing and handling of passing rent
</commit_message>
<xml_diff>
--- a/backend/data/templates/financial_model_template.xlsx
+++ b/backend/data/templates/financial_model_template.xlsx
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>82.87679999999999</v>
+        <v>85.44</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -634,7 +634,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>0.0485</v>
+        <v>0.0475</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -1336,7 +1336,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Logistics Corp A</t>
+          <t>Ingram Micro (UK) Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1345,29 +1345,29 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5000</v>
+        <v>222221</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2023-01-01</t>
+          <t>2015-06-01</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2028-12-31</t>
+          <t>2020-05-31</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>425000</v>
+        <v>1222215.5</v>
       </c>
       <c r="G2" t="n">
-        <v>85</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>E-Commerce Ltd</t>
+          <t>CNH Industrial N.V.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1376,23 +1376,23 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3000</v>
+        <v>90998</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2024-06-01</t>
+          <t>2002-11-19</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2029-05-31</t>
+          <t>2021-10-22</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>270000</v>
+        <v>409491</v>
       </c>
       <c r="G3" t="n">
-        <v>90</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="4">

</xml_diff>